<commit_message>
chore: add new TypeScript file and update layout component
- Added a new TypeScript file `hello.ts` with a simple console log statement.
- Updated the `layout.tsx` component to include an additional `<h1>` element.
- Removed an unused image file `image.png`.
- Updated binary Excel files with minor changes.
</commit_message>
<xml_diff>
--- a/117467240-3512564233.xlsx
+++ b/117467240-3512564233.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="16640"/>
+    <workbookView windowHeight="16160"/>
   </bookViews>
   <sheets>
     <sheet name="117467240-3512564233" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6063" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6059" uniqueCount="279">
   <si>
     <t>params</t>
   </si>
@@ -864,18 +864,6 @@
   </si>
   <si>
     <t>total_extension_count"":""238""}"</t>
-  </si>
-  <si>
-    <t>{"duration":"3073","enter_from":"setup","error_extension_count":"1","extension_result_list":"[\"alefragnani.project-manager-12.8.0-success\",\"Alibaba-Cloud.tongyi-lingma-1.4.12-skip\",\"Alibaba-Cloud.tongyi-lingma-1.4.13-success\",\"ChakrounAnas.turbo-console-log-2.10.5-success\",\"donjayamanne.githistory-0.6.20-success\",\"eamodio.gitlens-16.0.4-success\",\"ecmel.vscode-html-css-2.0.11-error\",\"formulahendry.auto-close-tag-0.5.15-success\",\"formulahendry.auto-rename-tag-0.1.10-success\",\"Gruntfuggly.todo-tree-0.0.226-success\",\"hollowtree.vue-snippets-1.0.4-success\",\"howardzuo.vscode-git-tags-1.4.4-success\",\"keraun.vue-beautify2-0.0.3-success\",\"octref.vetur-0.37.3-success\",\"pranaygp.vscode-css-peek-4.4.1-success\",\"shd101wyy.markdown-preview-enhanced-0.8.15-success\",\"skyran.js-jsx-snippets-11.1.3-success\",\"unifiedjs.vscode-mdx-1.8.11-success\",\"vincaslt.highlight-matching-tag-0.11.0-success\",\"yatki.vscode-surround-1.5.0-success\",\"zoo-team.zoo-vscode-extension-0.1.24-success\"]","is_success":"true","message":"","skip_extension_count":"1","success_extension_count":"19","total_extension_count":"21"}</t>
-  </si>
-  <si>
-    <t>{"duration":"10360","enter_from":"setup","error_extension_count":"25","extension_result_list":"[\"ant-codespaces.vscode-marketplace-1.0.0-success\",\"ant-codespaces.vscode-remote-1.2.0-error\",\"bungcip.better-toml-0.3.2-skip\",\"burkeholland.simple-react-snippets-1.2.8-success\",\"codeFuse.CodeFuse-2.4.0-success\",\"CoenraadS.bracket-pair-colorizer-2-0.2.4-success\",\"danields761.status-bar-breadcrumb-0.3.1-success\",\"dbaeumer.vscode-eslint-3.0.10-error\",\"donjayamanne.githistory-0.6.20-success\",\"dsznajder.es7-react-js-snippets-4.4.3-success\",\"dustypomerleau.rust-syntax-0.6.1-success\",\"eamodio.gitlens-16.0.4-success\",\"ecmel.vscode-html-css-2.0.11-error\",\"emmanuelbeziat.vscode-great-icons-2.1.111-skip\",\"esbenp.prettier-vscode-11.0.0-success\",\"evgeniypeshkov.syntax-highlighter-0.5.0-skip\",\"fabiospampinato.vscode-diff-2.1.2-error\",\"geddski.macros-1.2.1-success\",\"infeng.vscode-react-typescript-1.3.1-success\",\"JerryHong.autofilename-0.1.3-success\",\"JScearcy.rust-doc-viewer-4.2.0-success\",\"KevinRose.vsc-python-indent-1.18.0-success\",\"lextudio.restructuredtext-190.4.4-success\",\"lorenzopirro.rust-flash-snippets-3.1.1-success\",\"maggie.eslint-rules-zh-plugin-0.2.2-success\",\"mikey.vscode-fileheader-0.0.2-success\",\"mkxml.vscode-filesize-3.2.2-success\",\"ms-azuretools.vscode-docker-1.29.3-error\",\"ms-dotnettools.dotnet-interactive-vscode-1.0.5568010-error\",\"ms-python.debugpy-2024.12.0-error\",\"ms-python.isort-2023.10.1-error\",\"ms-python.pylint-2024.0.0-error\",\"ms-python.python-2024.14.1-skip\",\"ms-python.python-2024.16.0-skip\",\"ms-python.python-2024.16.1-skip\",\"ms-python.python-2024.18.0-skip\",\"ms-python.python-2024.18.1-skip\",\"ms-python.python-2024.20.0-skip\",\"ms-python.vscode-pylance-2024.11.3-error\",\"ms-toolsai.jupyter-2024.10.0-error\",\"ms-toolsai.jupyter-2024.7.0-error\",\"ms-toolsai.jupyter-2024.8.1-error\",\"ms-toolsai.jupyter-2024.9.1-error\",\"ms-toolsai.jupyter-keymap-1.1.2-success\",\"ms-toolsai.jupyter-renderers-1.0.19-success\",\"ms-toolsai.jupyter-renderers-1.0.21-error\",\"ms-toolsai.vscode-jupyter-cell-tags-0.1.9-error\",\"ms-toolsai.vscode-jupyter-slideshow-0.1.6-error\",\"ms-vscode-remote.remote-containers-0.388.0-error\",\"ms-vscode-remote.remote-ssh-0.115.1-error\",\"ms-vscode-remote.remote-ssh-edit-0.87.0-success\",\"ms-vscode-remote.remote-wsl-0.88.5-error\",\"ms-vscode-remote.vscode-remote-extensionpack-0.26.0-success\",\"ms-vscode.js-debug-nightly-2024.11.1917-skip\",\"ms-vscode.js-debug-nightly-2024.11.2917-success\",\"ms-vscode.remote-explorer-0.4.3-error\",\"ms-vscode.remote-server-1.5.2-error\",\"ms-vscode.sublime-keybindings-4.1.10-success\",\"niudai.vscode-zhihu-0.5.1-success\",\"nyxiative.rust-and-friends-1.0.0-skip\",\"octref.vetur-0.37.3-success\",\"PKief.material-icon-theme-5.14.1-skip\",\"PolyMeilex.rust-targets-1.1.1-success\",\"rbbit.typescript-hero-3.0.0-success\",\"redhat.java-1.36.0-skip\",\"redhat.java-1.37.0-success\",\"redhat.vscode-yaml-1.15.0-success\",\"ritwickdey.LiveServer-5.7.9-success\",\"ronnidc.nunjucks-0.3.1-success\",\"rust-lang.rust-analyzer-0.3.2196-skip\",\"rust-lang.rust-analyzer-0.3.2204-success\",\"serayuzgur.crates-0.6.7-skip\",\"statelyai.stately-vscode-2.1.0-success\",\"tamasfe.even-better-toml-0.19.2-success\",\"unifiedjs.vscode-mdx-1.8.11-success\",\"vadimcn.vscode-lldb-1.11.1-success\",\"VisualStudioExptTeam.intellicode-api-usage-examples-0.2.8-success\",\"VisualStudioExptTeam.intellicode-api-usage-examples-0.2.9-error\",\"VisualStudioExptTeam.vscodeintellicode-1.3.1-success\",\"VisualStudioExptTeam.vscodeintellicode-1.3.2-error\",\"vscjava.vscode-gradle-3.16.4-success\",\"vscjava.vscode-java-pack-0.29.0-success\",\"vscjava.vscode-maven-0.44.0-success\",\"waderyan.gitblame-11.1.1-error\",\"wix.vscode-import-cost-3.3.0-success\",\"xabikos.JavaScriptSnippets-1.8.0-success\",\"ZhangYue.rust-mod-generator-1.0.10-success\"]","is_success":"true","message":"","skip_extension_count":"15","success_extension_count":"47","total_extension_count":"87"}</t>
-  </si>
-  <si>
-    <t>{"duration":"3205","enter_from":"setup","error_extension_count":"7","extension_result_list":"[\"aaron-bond.better-comments-3.0.2-success\",\"anseki.vscode-color-0.4.5-success\",\"cesium.gltf-vscode-2.5.1-success\",\"christian-kohler.path-intellisense-2.10.0-success\",\"dbaeumer.vscode-eslint-3.0.10-error\",\"dlhtx.uniapp-snippet-0.0.2-success\",\"donjayamanne.githistory-0.6.20-success\",\"eamodio.gitlens-16.0.4-success\",\"ecmel.vscode-html-css-2.0.11-error\",\"Equinusocio.vsc-community-material-theme-1.4.7-skip\",\"Equinusocio.vsc-material-theme-34.7.9-skip\",\"esbenp.prettier-vscode-11.0.0-success\",\"formulahendry.auto-close-tag-0.5.15-success\",\"formulahendry.auto-rename-tag-0.1.10-success\",\"Gruntfuggly.todo-tree-0.0.226-success\",\"jock.svg-1.5.4-success\",\"k--kato.intellij-idea-keybindings-1.7.2-error\",\"k--kato.intellij-idea-keybindings-1.7.3-error\",\"MarsCode.marscode-extension-1.1.30-skip\",\"ms-python.debugpy-2024.12.0-error\",\"ms-python.python-2024.14.1-skip\",\"ms-python.python-2024.20.0-skip\",\"ms-python.vscode-pylance-2024.11.3-error\",\"ms-vscode.cmake-tools-1.19.52-success\",\"ms-vscode.cpptools-1.22.11-success\",\"naumovs.color-highlight-2.8.0-success\",\"octref.vetur-0.37.3-success\",\"PKief.material-icon-theme-5.14.1-skip\",\"pranaygp.vscode-css-peek-4.4.1-success\",\"redhat.vscode-xml-0.27.2-success\",\"ritwickdey.LiveServer-5.7.9-success\",\"russell.any-rule-0.3.18-success\",\"TabNine.tabnine-vscode-3.199.0-success\",\"twxs.cmake-0.0.17-success\",\"uni-helper.uni-app-schemas-vscode-0.9.3-success\",\"uni-helper.uni-app-snippets-vscode-0.10.5-success\",\"uni-helper.uni-cloud-snippets-vscode-0.3.0-success\",\"uni-helper.uni-helper-vscode-0.5.9-success\",\"uni-helper.uni-highlight-vscode-0.3.11-success\",\"uni-helper.uni-ui-snippets-vscode-0.6.6-success\",\"Vue.volar-2.0.8-success\",\"Vue.volar-2.1.10-error\",\"wayou.vscode-todo-highlight-1.0.5-success\",\"xabikos.JavaScriptSnippets-1.8.0-success\",\"yandeu.five-server-0.3.1-success\",\"yzhang.markdown-all-in-one-3.6.2-success\"]","is_success":"true","message":"","skip_extension_count":"5","success_extension_count":"33","total_extension_count":"45"}</t>
-  </si>
-  <si>
-    <t>{"duration":"2452","enter_from":"setup","error_extension_count":"15","extension_result_list":"[\"1YiB.rust-bundle-1.0.0-success\",\"CristianoBattini.maui-view-generator-0.0.1-error\",\"digitalboy.view-code-behind-1.0.1-error\",\"dustypomerleau.rust-syntax-0.6.1-success\",\"GitHub.codespaces-1.17.3-error\",\"in4margaret.compareit-0.0.2-success\",\"mechatroner.rainbow-csv-3.12.0-success\",\"mechatroner.rainbow-csv-3.13.0-error\",\"mhutchie.git-graph-1.30.0-success\",\"MS-CEINTL.vscode-language-pack-zh-hans-1.95.2024103009-skip\",\"ms-dotnettools.csdevkit-1.11.14-error\",\"ms-dotnettools.csdevkit-1.13.9-error\",\"ms-dotnettools.csharp-2.50.27-success\",\"ms-dotnettools.csharp-2.55.29-error\",\"ms-dotnettools.dotnet-maui-1.5.34-error\",\"ms-dotnettools.vscode-dotnet-runtime-2.2.3-success\",\"ms-python.debugpy-2024.12.0-error\",\"ms-python.python-2024.14.1-skip\",\"ms-python.python-2024.16.1-skip\",\"ms-python.python-2024.20.0-skip\",\"ms-python.vscode-pylance-2024.11.3-error\",\"ms-vscode-remote.remote-ssh-0.113.1-error\",\"ms-vscode-remote.remote-ssh-0.115.0-error\",\"ms-vscode-remote.remote-ssh-0.115.1-error\",\"ms-vscode-remote.remote-ssh-edit-0.87.0-success\",\"ms-vscode.remote-explorer-0.4.3-error\",\"rust-lang.rust-analyzer-0.3.2196-skip\",\"rust-lang.rust-analyzer-0.3.2204-success\",\"TelerikInc.telerik-maui-productivity-tools-1.4.0-error\"]","is_success":"true","message":"","skip_extension_count":"5","success_extension_count":"9","total_extension_count":"29"}</t>
   </si>
 </sst>
 </file>
@@ -2028,7 +2016,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:ELX31"/>
+  <dimension ref="A1:ELX27"/>
   <sheetFormatPr defaultColWidth="10.3846153846154" defaultRowHeight="16.8"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -20260,26 +20248,6 @@
       </c>
       <c r="ELX27" t="s">
         <v>278</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1">
-      <c r="A28" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1">
-      <c r="A29" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1">
-      <c r="A30" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1">
-      <c r="A31" t="s">
-        <v>282</v>
       </c>
     </row>
   </sheetData>

</xml_diff>